<commit_message>
V3.14.04.2026.01 - Added Sequence Diagram and Flow Chart
</commit_message>
<xml_diff>
--- a/Documentation/Security Matrix V1.0.xlsx
+++ b/Documentation/Security Matrix V1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ahmed\Desktop\EA\2026\Personal\CC\Pre-Development\Documentation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Change-Control-HTML-Design\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C07980C2-32E6-4FC8-B7E2-605DA41FC90F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -621,12 +621,30 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -647,24 +665,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1082,57 +1082,57 @@
   <sheetData>
     <row r="1" spans="2:56" s="1" customFormat="1" ht="4.2" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:56" ht="44.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
-      <c r="AA2" s="23"/>
-      <c r="AB2" s="23"/>
-      <c r="AC2" s="23"/>
-      <c r="AD2" s="23"/>
-      <c r="AE2" s="23"/>
-      <c r="AF2" s="23"/>
-      <c r="AG2" s="23"/>
-      <c r="AH2" s="23"/>
-      <c r="AI2" s="23"/>
-      <c r="AJ2" s="23"/>
-      <c r="AK2" s="23"/>
-      <c r="AL2" s="23"/>
-      <c r="AM2" s="23"/>
-      <c r="AN2" s="23"/>
-      <c r="AO2" s="23"/>
-      <c r="AP2" s="23"/>
-      <c r="AQ2" s="23"/>
-      <c r="AR2" s="23"/>
-      <c r="AS2" s="23"/>
-      <c r="AT2" s="23"/>
-      <c r="AU2" s="23"/>
-      <c r="AV2" s="23"/>
-      <c r="AW2" s="23"/>
-      <c r="AX2" s="23"/>
-      <c r="AY2" s="23"/>
-      <c r="AZ2" s="23"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+      <c r="P2" s="29"/>
+      <c r="Q2" s="29"/>
+      <c r="R2" s="29"/>
+      <c r="S2" s="29"/>
+      <c r="T2" s="29"/>
+      <c r="U2" s="29"/>
+      <c r="V2" s="29"/>
+      <c r="W2" s="29"/>
+      <c r="X2" s="29"/>
+      <c r="Y2" s="29"/>
+      <c r="Z2" s="29"/>
+      <c r="AA2" s="29"/>
+      <c r="AB2" s="29"/>
+      <c r="AC2" s="29"/>
+      <c r="AD2" s="29"/>
+      <c r="AE2" s="29"/>
+      <c r="AF2" s="29"/>
+      <c r="AG2" s="29"/>
+      <c r="AH2" s="29"/>
+      <c r="AI2" s="29"/>
+      <c r="AJ2" s="29"/>
+      <c r="AK2" s="29"/>
+      <c r="AL2" s="29"/>
+      <c r="AM2" s="29"/>
+      <c r="AN2" s="29"/>
+      <c r="AO2" s="29"/>
+      <c r="AP2" s="29"/>
+      <c r="AQ2" s="29"/>
+      <c r="AR2" s="29"/>
+      <c r="AS2" s="29"/>
+      <c r="AT2" s="29"/>
+      <c r="AU2" s="29"/>
+      <c r="AV2" s="29"/>
+      <c r="AW2" s="29"/>
+      <c r="AX2" s="29"/>
+      <c r="AY2" s="29"/>
+      <c r="AZ2" s="29"/>
     </row>
     <row r="3" spans="2:56" ht="147.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="10"/>
@@ -1292,128 +1292,128 @@
     <row r="4" spans="2:56" s="14" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="12"/>
       <c r="C4" s="13"/>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="24"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24"/>
-      <c r="J4" s="24"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="24"/>
-      <c r="N4" s="24"/>
-      <c r="O4" s="24"/>
-      <c r="P4" s="24"/>
-      <c r="Q4" s="24"/>
-      <c r="R4" s="24"/>
-      <c r="S4" s="24"/>
-      <c r="T4" s="25" t="s">
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
+      <c r="I4" s="30"/>
+      <c r="J4" s="30"/>
+      <c r="K4" s="30"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="30"/>
+      <c r="N4" s="30"/>
+      <c r="O4" s="30"/>
+      <c r="P4" s="30"/>
+      <c r="Q4" s="30"/>
+      <c r="R4" s="30"/>
+      <c r="S4" s="30"/>
+      <c r="T4" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="U4" s="25"/>
-      <c r="V4" s="25"/>
-      <c r="W4" s="25"/>
-      <c r="X4" s="25"/>
-      <c r="Y4" s="25"/>
-      <c r="Z4" s="25"/>
-      <c r="AA4" s="25"/>
-      <c r="AB4" s="28" t="s">
+      <c r="U4" s="31"/>
+      <c r="V4" s="31"/>
+      <c r="W4" s="31"/>
+      <c r="X4" s="31"/>
+      <c r="Y4" s="31"/>
+      <c r="Z4" s="31"/>
+      <c r="AA4" s="31"/>
+      <c r="AB4" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="AC4" s="28"/>
-      <c r="AD4" s="28"/>
-      <c r="AE4" s="28"/>
-      <c r="AF4" s="29" t="s">
+      <c r="AC4" s="34"/>
+      <c r="AD4" s="34"/>
+      <c r="AE4" s="34"/>
+      <c r="AF4" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="AG4" s="29"/>
-      <c r="AH4" s="29"/>
-      <c r="AI4" s="29"/>
-      <c r="AJ4" s="29"/>
-      <c r="AK4" s="29"/>
-      <c r="AL4" s="30" t="s">
+      <c r="AG4" s="35"/>
+      <c r="AH4" s="35"/>
+      <c r="AI4" s="35"/>
+      <c r="AJ4" s="35"/>
+      <c r="AK4" s="35"/>
+      <c r="AL4" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="AM4" s="31"/>
-      <c r="AN4" s="31"/>
-      <c r="AO4" s="31"/>
-      <c r="AP4" s="31"/>
-      <c r="AQ4" s="31"/>
-      <c r="AR4" s="31"/>
-      <c r="AS4" s="31"/>
-      <c r="AT4" s="31"/>
-      <c r="AU4" s="31"/>
-      <c r="AV4" s="31"/>
-      <c r="AW4" s="31"/>
-      <c r="AX4" s="32"/>
+      <c r="AM4" s="26"/>
+      <c r="AN4" s="26"/>
+      <c r="AO4" s="26"/>
+      <c r="AP4" s="26"/>
+      <c r="AQ4" s="26"/>
+      <c r="AR4" s="26"/>
+      <c r="AS4" s="26"/>
+      <c r="AT4" s="26"/>
+      <c r="AU4" s="26"/>
+      <c r="AV4" s="26"/>
+      <c r="AW4" s="26"/>
+      <c r="AX4" s="27"/>
       <c r="AY4" s="20"/>
       <c r="AZ4" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="34"/>
-      <c r="M5" s="34"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="34"/>
-      <c r="P5" s="34"/>
-      <c r="Q5" s="34"/>
-      <c r="R5" s="34"/>
-      <c r="S5" s="34"/>
-      <c r="T5" s="34"/>
-      <c r="U5" s="34"/>
-      <c r="V5" s="34"/>
-      <c r="W5" s="34"/>
-      <c r="X5" s="34"/>
-      <c r="Y5" s="34"/>
-      <c r="Z5" s="34"/>
-      <c r="AA5" s="34"/>
-      <c r="AB5" s="34"/>
-      <c r="AC5" s="34"/>
-      <c r="AD5" s="34"/>
-      <c r="AE5" s="34"/>
-      <c r="AF5" s="34"/>
-      <c r="AG5" s="34"/>
-      <c r="AH5" s="34"/>
-      <c r="AI5" s="34"/>
-      <c r="AJ5" s="34"/>
-      <c r="AK5" s="34"/>
-      <c r="AL5" s="34"/>
-      <c r="AM5" s="34"/>
-      <c r="AN5" s="34"/>
-      <c r="AO5" s="34"/>
-      <c r="AP5" s="34"/>
-      <c r="AQ5" s="34"/>
-      <c r="AR5" s="34"/>
-      <c r="AS5" s="34"/>
-      <c r="AT5" s="34"/>
-      <c r="AU5" s="34"/>
-      <c r="AV5" s="34"/>
-      <c r="AW5" s="34"/>
-      <c r="AX5" s="34"/>
-      <c r="AY5" s="34"/>
-      <c r="AZ5" s="35"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="22"/>
+      <c r="V5" s="22"/>
+      <c r="W5" s="22"/>
+      <c r="X5" s="22"/>
+      <c r="Y5" s="22"/>
+      <c r="Z5" s="22"/>
+      <c r="AA5" s="22"/>
+      <c r="AB5" s="22"/>
+      <c r="AC5" s="22"/>
+      <c r="AD5" s="22"/>
+      <c r="AE5" s="22"/>
+      <c r="AF5" s="22"/>
+      <c r="AG5" s="22"/>
+      <c r="AH5" s="22"/>
+      <c r="AI5" s="22"/>
+      <c r="AJ5" s="22"/>
+      <c r="AK5" s="22"/>
+      <c r="AL5" s="22"/>
+      <c r="AM5" s="22"/>
+      <c r="AN5" s="22"/>
+      <c r="AO5" s="22"/>
+      <c r="AP5" s="22"/>
+      <c r="AQ5" s="22"/>
+      <c r="AR5" s="22"/>
+      <c r="AS5" s="22"/>
+      <c r="AT5" s="22"/>
+      <c r="AU5" s="22"/>
+      <c r="AV5" s="22"/>
+      <c r="AW5" s="22"/>
+      <c r="AX5" s="22"/>
+      <c r="AY5" s="22"/>
+      <c r="AZ5" s="23"/>
     </row>
     <row r="6" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="22"/>
+      <c r="C6" s="24"/>
       <c r="D6" s="17"/>
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
@@ -1465,10 +1465,10 @@
       <c r="AZ6" s="18"/>
     </row>
     <row r="7" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="22"/>
+      <c r="C7" s="24"/>
       <c r="D7" s="17"/>
       <c r="E7" s="17"/>
       <c r="F7" s="17"/>
@@ -1520,10 +1520,10 @@
       <c r="AZ7" s="17"/>
     </row>
     <row r="8" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="22"/>
+      <c r="C8" s="24"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
       <c r="F8" s="17"/>
@@ -1575,10 +1575,10 @@
       <c r="AZ8" s="17"/>
     </row>
     <row r="9" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="22"/>
+      <c r="C9" s="24"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
       <c r="F9" s="17"/>
@@ -1630,65 +1630,65 @@
       <c r="AZ9" s="17"/>
     </row>
     <row r="10" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="34"/>
-      <c r="T10" s="34"/>
-      <c r="U10" s="34"/>
-      <c r="V10" s="34"/>
-      <c r="W10" s="34"/>
-      <c r="X10" s="34"/>
-      <c r="Y10" s="34"/>
-      <c r="Z10" s="34"/>
-      <c r="AA10" s="34"/>
-      <c r="AB10" s="34"/>
-      <c r="AC10" s="34"/>
-      <c r="AD10" s="34"/>
-      <c r="AE10" s="34"/>
-      <c r="AF10" s="34"/>
-      <c r="AG10" s="34"/>
-      <c r="AH10" s="34"/>
-      <c r="AI10" s="34"/>
-      <c r="AJ10" s="34"/>
-      <c r="AK10" s="34"/>
-      <c r="AL10" s="34"/>
-      <c r="AM10" s="34"/>
-      <c r="AN10" s="34"/>
-      <c r="AO10" s="34"/>
-      <c r="AP10" s="34"/>
-      <c r="AQ10" s="34"/>
-      <c r="AR10" s="34"/>
-      <c r="AS10" s="34"/>
-      <c r="AT10" s="34"/>
-      <c r="AU10" s="34"/>
-      <c r="AV10" s="34"/>
-      <c r="AW10" s="34"/>
-      <c r="AX10" s="34"/>
-      <c r="AY10" s="34"/>
-      <c r="AZ10" s="35"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22"/>
+      <c r="T10" s="22"/>
+      <c r="U10" s="22"/>
+      <c r="V10" s="22"/>
+      <c r="W10" s="22"/>
+      <c r="X10" s="22"/>
+      <c r="Y10" s="22"/>
+      <c r="Z10" s="22"/>
+      <c r="AA10" s="22"/>
+      <c r="AB10" s="22"/>
+      <c r="AC10" s="22"/>
+      <c r="AD10" s="22"/>
+      <c r="AE10" s="22"/>
+      <c r="AF10" s="22"/>
+      <c r="AG10" s="22"/>
+      <c r="AH10" s="22"/>
+      <c r="AI10" s="22"/>
+      <c r="AJ10" s="22"/>
+      <c r="AK10" s="22"/>
+      <c r="AL10" s="22"/>
+      <c r="AM10" s="22"/>
+      <c r="AN10" s="22"/>
+      <c r="AO10" s="22"/>
+      <c r="AP10" s="22"/>
+      <c r="AQ10" s="22"/>
+      <c r="AR10" s="22"/>
+      <c r="AS10" s="22"/>
+      <c r="AT10" s="22"/>
+      <c r="AU10" s="22"/>
+      <c r="AV10" s="22"/>
+      <c r="AW10" s="22"/>
+      <c r="AX10" s="22"/>
+      <c r="AY10" s="22"/>
+      <c r="AZ10" s="23"/>
     </row>
     <row r="11" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C11" s="22"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>
@@ -1740,10 +1740,10 @@
       <c r="AZ11" s="17"/>
     </row>
     <row r="12" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="22"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="17"/>
       <c r="E12" s="17"/>
       <c r="F12" s="17"/>
@@ -1795,10 +1795,10 @@
       <c r="AZ12" s="17"/>
     </row>
     <row r="13" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C13" s="22"/>
+      <c r="C13" s="24"/>
       <c r="D13" s="17"/>
       <c r="E13" s="17"/>
       <c r="F13" s="17"/>
@@ -1850,10 +1850,10 @@
       <c r="AZ13" s="17"/>
     </row>
     <row r="14" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="22"/>
+      <c r="C14" s="24"/>
       <c r="D14" s="17"/>
       <c r="E14" s="17"/>
       <c r="F14" s="17"/>
@@ -1905,65 +1905,65 @@
       <c r="AZ14" s="17"/>
     </row>
     <row r="15" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="34"/>
-      <c r="H15" s="34"/>
-      <c r="I15" s="34"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
-      <c r="M15" s="34"/>
-      <c r="N15" s="34"/>
-      <c r="O15" s="34"/>
-      <c r="P15" s="34"/>
-      <c r="Q15" s="34"/>
-      <c r="R15" s="34"/>
-      <c r="S15" s="34"/>
-      <c r="T15" s="34"/>
-      <c r="U15" s="34"/>
-      <c r="V15" s="34"/>
-      <c r="W15" s="34"/>
-      <c r="X15" s="34"/>
-      <c r="Y15" s="34"/>
-      <c r="Z15" s="34"/>
-      <c r="AA15" s="34"/>
-      <c r="AB15" s="34"/>
-      <c r="AC15" s="34"/>
-      <c r="AD15" s="34"/>
-      <c r="AE15" s="34"/>
-      <c r="AF15" s="34"/>
-      <c r="AG15" s="34"/>
-      <c r="AH15" s="34"/>
-      <c r="AI15" s="34"/>
-      <c r="AJ15" s="34"/>
-      <c r="AK15" s="34"/>
-      <c r="AL15" s="34"/>
-      <c r="AM15" s="34"/>
-      <c r="AN15" s="34"/>
-      <c r="AO15" s="34"/>
-      <c r="AP15" s="34"/>
-      <c r="AQ15" s="34"/>
-      <c r="AR15" s="34"/>
-      <c r="AS15" s="34"/>
-      <c r="AT15" s="34"/>
-      <c r="AU15" s="34"/>
-      <c r="AV15" s="34"/>
-      <c r="AW15" s="34"/>
-      <c r="AX15" s="34"/>
-      <c r="AY15" s="34"/>
-      <c r="AZ15" s="35"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+      <c r="J15" s="22"/>
+      <c r="K15" s="22"/>
+      <c r="L15" s="22"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
+      <c r="P15" s="22"/>
+      <c r="Q15" s="22"/>
+      <c r="R15" s="22"/>
+      <c r="S15" s="22"/>
+      <c r="T15" s="22"/>
+      <c r="U15" s="22"/>
+      <c r="V15" s="22"/>
+      <c r="W15" s="22"/>
+      <c r="X15" s="22"/>
+      <c r="Y15" s="22"/>
+      <c r="Z15" s="22"/>
+      <c r="AA15" s="22"/>
+      <c r="AB15" s="22"/>
+      <c r="AC15" s="22"/>
+      <c r="AD15" s="22"/>
+      <c r="AE15" s="22"/>
+      <c r="AF15" s="22"/>
+      <c r="AG15" s="22"/>
+      <c r="AH15" s="22"/>
+      <c r="AI15" s="22"/>
+      <c r="AJ15" s="22"/>
+      <c r="AK15" s="22"/>
+      <c r="AL15" s="22"/>
+      <c r="AM15" s="22"/>
+      <c r="AN15" s="22"/>
+      <c r="AO15" s="22"/>
+      <c r="AP15" s="22"/>
+      <c r="AQ15" s="22"/>
+      <c r="AR15" s="22"/>
+      <c r="AS15" s="22"/>
+      <c r="AT15" s="22"/>
+      <c r="AU15" s="22"/>
+      <c r="AV15" s="22"/>
+      <c r="AW15" s="22"/>
+      <c r="AX15" s="22"/>
+      <c r="AY15" s="22"/>
+      <c r="AZ15" s="23"/>
     </row>
     <row r="16" spans="2:56" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="22"/>
+      <c r="C16" s="24"/>
       <c r="D16" s="17"/>
       <c r="E16" s="17"/>
       <c r="F16" s="17"/>
@@ -2015,10 +2015,10 @@
       <c r="AZ16" s="17"/>
     </row>
     <row r="17" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="22"/>
+      <c r="C17" s="24"/>
       <c r="D17" s="17"/>
       <c r="E17" s="17"/>
       <c r="F17" s="17"/>
@@ -2070,10 +2070,10 @@
       <c r="AZ17" s="17"/>
     </row>
     <row r="18" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="22"/>
+      <c r="C18" s="24"/>
       <c r="D18" s="17"/>
       <c r="E18" s="17"/>
       <c r="F18" s="17"/>
@@ -2125,10 +2125,10 @@
       <c r="AZ18" s="17"/>
     </row>
     <row r="19" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="22"/>
+      <c r="C19" s="24"/>
       <c r="D19" s="17"/>
       <c r="E19" s="17"/>
       <c r="F19" s="17"/>
@@ -2180,65 +2180,65 @@
       <c r="AZ19" s="17"/>
     </row>
     <row r="20" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C20" s="21"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="34"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
-      <c r="P20" s="34"/>
-      <c r="Q20" s="34"/>
-      <c r="R20" s="34"/>
-      <c r="S20" s="34"/>
-      <c r="T20" s="34"/>
-      <c r="U20" s="34"/>
-      <c r="V20" s="34"/>
-      <c r="W20" s="34"/>
-      <c r="X20" s="34"/>
-      <c r="Y20" s="34"/>
-      <c r="Z20" s="34"/>
-      <c r="AA20" s="34"/>
-      <c r="AB20" s="34"/>
-      <c r="AC20" s="34"/>
-      <c r="AD20" s="34"/>
-      <c r="AE20" s="34"/>
-      <c r="AF20" s="34"/>
-      <c r="AG20" s="34"/>
-      <c r="AH20" s="34"/>
-      <c r="AI20" s="34"/>
-      <c r="AJ20" s="34"/>
-      <c r="AK20" s="34"/>
-      <c r="AL20" s="34"/>
-      <c r="AM20" s="34"/>
-      <c r="AN20" s="34"/>
-      <c r="AO20" s="34"/>
-      <c r="AP20" s="34"/>
-      <c r="AQ20" s="34"/>
-      <c r="AR20" s="34"/>
-      <c r="AS20" s="34"/>
-      <c r="AT20" s="34"/>
-      <c r="AU20" s="34"/>
-      <c r="AV20" s="34"/>
-      <c r="AW20" s="34"/>
-      <c r="AX20" s="34"/>
-      <c r="AY20" s="34"/>
-      <c r="AZ20" s="35"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="22"/>
+      <c r="Q20" s="22"/>
+      <c r="R20" s="22"/>
+      <c r="S20" s="22"/>
+      <c r="T20" s="22"/>
+      <c r="U20" s="22"/>
+      <c r="V20" s="22"/>
+      <c r="W20" s="22"/>
+      <c r="X20" s="22"/>
+      <c r="Y20" s="22"/>
+      <c r="Z20" s="22"/>
+      <c r="AA20" s="22"/>
+      <c r="AB20" s="22"/>
+      <c r="AC20" s="22"/>
+      <c r="AD20" s="22"/>
+      <c r="AE20" s="22"/>
+      <c r="AF20" s="22"/>
+      <c r="AG20" s="22"/>
+      <c r="AH20" s="22"/>
+      <c r="AI20" s="22"/>
+      <c r="AJ20" s="22"/>
+      <c r="AK20" s="22"/>
+      <c r="AL20" s="22"/>
+      <c r="AM20" s="22"/>
+      <c r="AN20" s="22"/>
+      <c r="AO20" s="22"/>
+      <c r="AP20" s="22"/>
+      <c r="AQ20" s="22"/>
+      <c r="AR20" s="22"/>
+      <c r="AS20" s="22"/>
+      <c r="AT20" s="22"/>
+      <c r="AU20" s="22"/>
+      <c r="AV20" s="22"/>
+      <c r="AW20" s="22"/>
+      <c r="AX20" s="22"/>
+      <c r="AY20" s="22"/>
+      <c r="AZ20" s="23"/>
     </row>
     <row r="21" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="22"/>
+      <c r="C21" s="24"/>
       <c r="D21" s="17"/>
       <c r="E21" s="17"/>
       <c r="F21" s="17"/>
@@ -2290,10 +2290,10 @@
       <c r="AZ21" s="17"/>
     </row>
     <row r="22" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C22" s="22"/>
+      <c r="C22" s="24"/>
       <c r="D22" s="17"/>
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
@@ -2345,10 +2345,10 @@
       <c r="AZ22" s="17"/>
     </row>
     <row r="23" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C23" s="22"/>
+      <c r="C23" s="24"/>
       <c r="D23" s="17"/>
       <c r="E23" s="17"/>
       <c r="F23" s="17"/>
@@ -2400,10 +2400,10 @@
       <c r="AZ23" s="17"/>
     </row>
     <row r="24" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C24" s="22"/>
+      <c r="C24" s="24"/>
       <c r="D24" s="17"/>
       <c r="E24" s="17"/>
       <c r="F24" s="17"/>
@@ -2455,65 +2455,65 @@
       <c r="AZ24" s="17"/>
     </row>
     <row r="25" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="34"/>
-      <c r="H25" s="34"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
-      <c r="M25" s="34"/>
-      <c r="N25" s="34"/>
-      <c r="O25" s="34"/>
-      <c r="P25" s="34"/>
-      <c r="Q25" s="34"/>
-      <c r="R25" s="34"/>
-      <c r="S25" s="34"/>
-      <c r="T25" s="34"/>
-      <c r="U25" s="34"/>
-      <c r="V25" s="34"/>
-      <c r="W25" s="34"/>
-      <c r="X25" s="34"/>
-      <c r="Y25" s="34"/>
-      <c r="Z25" s="34"/>
-      <c r="AA25" s="34"/>
-      <c r="AB25" s="34"/>
-      <c r="AC25" s="34"/>
-      <c r="AD25" s="34"/>
-      <c r="AE25" s="34"/>
-      <c r="AF25" s="34"/>
-      <c r="AG25" s="34"/>
-      <c r="AH25" s="34"/>
-      <c r="AI25" s="34"/>
-      <c r="AJ25" s="34"/>
-      <c r="AK25" s="34"/>
-      <c r="AL25" s="34"/>
-      <c r="AM25" s="34"/>
-      <c r="AN25" s="34"/>
-      <c r="AO25" s="34"/>
-      <c r="AP25" s="34"/>
-      <c r="AQ25" s="34"/>
-      <c r="AR25" s="34"/>
-      <c r="AS25" s="34"/>
-      <c r="AT25" s="34"/>
-      <c r="AU25" s="34"/>
-      <c r="AV25" s="34"/>
-      <c r="AW25" s="34"/>
-      <c r="AX25" s="34"/>
-      <c r="AY25" s="34"/>
-      <c r="AZ25" s="35"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="22"/>
+      <c r="Q25" s="22"/>
+      <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
+      <c r="T25" s="22"/>
+      <c r="U25" s="22"/>
+      <c r="V25" s="22"/>
+      <c r="W25" s="22"/>
+      <c r="X25" s="22"/>
+      <c r="Y25" s="22"/>
+      <c r="Z25" s="22"/>
+      <c r="AA25" s="22"/>
+      <c r="AB25" s="22"/>
+      <c r="AC25" s="22"/>
+      <c r="AD25" s="22"/>
+      <c r="AE25" s="22"/>
+      <c r="AF25" s="22"/>
+      <c r="AG25" s="22"/>
+      <c r="AH25" s="22"/>
+      <c r="AI25" s="22"/>
+      <c r="AJ25" s="22"/>
+      <c r="AK25" s="22"/>
+      <c r="AL25" s="22"/>
+      <c r="AM25" s="22"/>
+      <c r="AN25" s="22"/>
+      <c r="AO25" s="22"/>
+      <c r="AP25" s="22"/>
+      <c r="AQ25" s="22"/>
+      <c r="AR25" s="22"/>
+      <c r="AS25" s="22"/>
+      <c r="AT25" s="22"/>
+      <c r="AU25" s="22"/>
+      <c r="AV25" s="22"/>
+      <c r="AW25" s="22"/>
+      <c r="AX25" s="22"/>
+      <c r="AY25" s="22"/>
+      <c r="AZ25" s="23"/>
     </row>
     <row r="26" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="22"/>
+      <c r="C26" s="24"/>
       <c r="D26" s="17"/>
       <c r="E26" s="17"/>
       <c r="F26" s="17"/>
@@ -2565,10 +2565,10 @@
       <c r="AZ26" s="17"/>
     </row>
     <row r="27" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="22"/>
+      <c r="C27" s="24"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
       <c r="F27" s="17"/>
@@ -2620,10 +2620,10 @@
       <c r="AZ27" s="17"/>
     </row>
     <row r="28" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="22"/>
+      <c r="C28" s="24"/>
       <c r="D28" s="17"/>
       <c r="E28" s="17"/>
       <c r="F28" s="17"/>
@@ -2675,10 +2675,10 @@
       <c r="AZ28" s="17"/>
     </row>
     <row r="29" spans="2:52" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="22"/>
+      <c r="C29" s="24"/>
       <c r="D29" s="17"/>
       <c r="E29" s="17"/>
       <c r="F29" s="17"/>
@@ -2757,30 +2757,6 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="D25:AZ25"/>
-    <mergeCell ref="D20:AZ20"/>
-    <mergeCell ref="D15:AZ15"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="AL4:AX4"/>
-    <mergeCell ref="D5:AZ5"/>
-    <mergeCell ref="D10:AZ10"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B2:AZ2"/>
-    <mergeCell ref="D4:S4"/>
-    <mergeCell ref="T4:AA4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="AB4:AE4"/>
-    <mergeCell ref="AF4:AK4"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
@@ -2794,6 +2770,30 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B2:AZ2"/>
+    <mergeCell ref="D4:S4"/>
+    <mergeCell ref="T4:AA4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="AB4:AE4"/>
+    <mergeCell ref="AF4:AK4"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="AL4:AX4"/>
+    <mergeCell ref="D5:AZ5"/>
+    <mergeCell ref="D10:AZ10"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D25:AZ25"/>
+    <mergeCell ref="D20:AZ20"/>
+    <mergeCell ref="D15:AZ15"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.4" bottom="0.4" header="0" footer="0"/>
   <pageSetup scale="70" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>